<commit_message>
feat: apply full Sales Won audit reclassifications (28 Net New / 140 Upsell / 36 Renewal)
Resale (29) + Other (37) → Upsell (product subscriptions / existing-client add-ons)
Imagine Columbus Primary Academy Renewal → Upsell (new service confirmed in Power BI)
21 deals across 15 clients → Net New (Power BI REST API: MIN(StartDate) 2025+,
  dataset 5ee15556); nnClients var added to renderSalesWon()
Net New KPI: "20 new logos · Jan 2025–Feb 2026"; footer cites Power BI API
XLSX All Deals Detail col C+J updated to match; Is Growth? column corrected

Result: 28 Net New / 140 Upsell / 36 Renewal = 204 deals · $335,103/mo · 20 logos

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Sales Won Audit - MRR Analysis.xlsx
+++ b/Sales Won Audit - MRR Analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Deals Detail" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Sales Rep" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Renewals Detail" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="All Deals Detail" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="By Sales Rep" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Renewals Detail" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Deals Detail'!$A$1:$J$205</definedName>

</xml_diff>